<commit_message>
added some plots capabilities
</commit_message>
<xml_diff>
--- a/lcoe_plots/synthetic_ethylene_lcoe/LCOE_SYNTHETIC_Ethylene.xlsx
+++ b/lcoe_plots/synthetic_ethylene_lcoe/LCOE_SYNTHETIC_Ethylene.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/abbie/MacroEnergy-Abbie.jl/MacroEnergyExamples/lcoe_plots/synthetic_ethylene_lcoe/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FFCDA25-4E66-5C49-AB40-1F00B1ECA7A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DB35CF9-A81C-D44E-9ABF-AAB53455FB4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="17740" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="17740" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="lc_detailed" sheetId="1" r:id="rId1"/>
-    <sheet name="lc_summary" sheetId="2" r:id="rId2"/>
+    <sheet name="lc_summary_noseq" sheetId="2" r:id="rId2"/>
+    <sheet name="lc_summary_seq" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="95">
   <si>
     <t>Asset Parameters (normalized by commodity feedstock)</t>
   </si>
@@ -198,7 +199,7 @@
     <t>elec_consumption</t>
   </si>
   <si>
-    <t>ethane_consumption</t>
+    <t>co2captured_consumption</t>
   </si>
   <si>
     <t>natgas_production</t>
@@ -270,7 +271,7 @@
     <t>t-CO2/t-ethylene</t>
   </si>
   <si>
-    <t>Synthetic_Ethylene_Non_CCS</t>
+    <t>SE_Synthetic_Ethylene_Non_CCS</t>
   </si>
   <si>
     <t>CO2Captured</t>
@@ -282,7 +283,7 @@
     <t>t-CO2/MWh-gasoline</t>
   </si>
   <si>
-    <t>Synthetic_Ethylene_CCS_90</t>
+    <t>SE_Synthetic_Ethylene_CCS_90</t>
   </si>
   <si>
     <t>Natural Gas Carbon Content</t>
@@ -303,22 +304,22 @@
     <t>%</t>
   </si>
   <si>
+    <t>Levelized cost for Synthetic Ethylene Production - $/GJ-ethylene - no chemicals CO2 sequestration</t>
+  </si>
+  <si>
     <t>LCOE ($/GJ-ethylene)</t>
   </si>
   <si>
-    <t>Levelized cost for Synthetic Ethylene Production - $/GJ-ethylene - no chemicals CO2 sequestration</t>
+    <t>CHECK LCOE ($/GJ-ethylene)</t>
+  </si>
+  <si>
+    <t>Ethylene LHV</t>
+  </si>
+  <si>
+    <t>GJ/t-ethylene</t>
   </si>
   <si>
     <t>Levelized cost for Synthetic Ethylene Production - $/GJ-ethylene - chemicals CO2 sequestration</t>
-  </si>
-  <si>
-    <t>Ethylene LHV</t>
-  </si>
-  <si>
-    <t>GJ/t-ethylene</t>
-  </si>
-  <si>
-    <t>CHECK LCOE ($/GJ-ethylene)</t>
   </si>
 </sst>
 </file>
@@ -915,8 +916,8 @@
     <col min="82" max="82" width="22.5" style="1" bestFit="1" customWidth="1"/>
     <col min="83" max="83" width="10.83203125" style="1" customWidth="1"/>
     <col min="84" max="84" width="17.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="85" max="92" width="10.83203125" style="1" customWidth="1"/>
-    <col min="93" max="16384" width="10.83203125" style="1"/>
+    <col min="85" max="95" width="10.83203125" style="1" customWidth="1"/>
+    <col min="96" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:84" x14ac:dyDescent="0.2">
@@ -1239,31 +1240,55 @@
       <c r="O4" s="16">
         <v>122.135409</v>
       </c>
-      <c r="P4" s="16"/>
-      <c r="Q4" s="16"/>
-      <c r="R4" s="16"/>
-      <c r="S4" s="16"/>
+      <c r="P4" s="16">
+        <v>-10.071578000000001</v>
+      </c>
+      <c r="Q4" s="16">
+        <v>73.297528</v>
+      </c>
+      <c r="R4" s="16">
+        <v>77.158259999999999</v>
+      </c>
+      <c r="S4" s="16">
+        <v>59.694023999999999</v>
+      </c>
       <c r="T4" s="11">
         <v>21.986353300000001</v>
       </c>
       <c r="U4" s="17"/>
       <c r="V4" s="17"/>
-      <c r="W4" s="16"/>
-      <c r="X4" s="16"/>
+      <c r="W4" s="16">
+        <v>26.556269</v>
+      </c>
+      <c r="X4" s="16">
+        <v>8.6278919999999992</v>
+      </c>
       <c r="Y4" s="16"/>
-      <c r="Z4" s="17"/>
-      <c r="AA4" s="17"/>
+      <c r="Z4" s="17">
+        <v>-96.133976000000004</v>
+      </c>
+      <c r="AA4" s="17">
+        <v>-96.133976000000004</v>
+      </c>
       <c r="AB4" s="17"/>
       <c r="AC4" s="17"/>
       <c r="AD4" s="17"/>
       <c r="AE4" s="17"/>
-      <c r="AF4" s="16"/>
-      <c r="AG4" s="16"/>
-      <c r="AH4" s="16"/>
-      <c r="AI4" s="16"/>
+      <c r="AF4" s="16">
+        <v>4.7546840000000001</v>
+      </c>
+      <c r="AG4" s="16">
+        <v>-0.13628299999999999</v>
+      </c>
+      <c r="AH4" s="16">
+        <v>576.81126900000004</v>
+      </c>
+      <c r="AI4" s="16">
+        <v>576.81126900000004</v>
+      </c>
       <c r="AK4" s="1" t="str">
         <f>B4</f>
-        <v>Synthetic_Ethylene_Non_CCS</v>
+        <v>SE_Synthetic_Ethylene_Non_CCS</v>
       </c>
       <c r="AL4" s="1" t="str">
         <f>C4</f>
@@ -1271,11 +1296,11 @@
       </c>
       <c r="AM4" s="12">
         <f>SUM(AS4:AZ4)+BB4+BC4</f>
-        <v>476.64414784303057</v>
+        <v>1069.5117340943755</v>
       </c>
       <c r="AN4" s="12">
         <f>SUM(AS4:AZ4)+BE4+BF4</f>
-        <v>476.64414784303057</v>
+        <v>1069.5117340943755</v>
       </c>
       <c r="AO4" s="5">
         <f>AM4-AN4</f>
@@ -1283,11 +1308,11 @@
       </c>
       <c r="AP4" s="12">
         <f>SUM(AS4:AZ4)+BH4+BI4</f>
-        <v>520.27386164750192</v>
+        <v>1113.1414478988468</v>
       </c>
       <c r="AQ4" s="12">
         <f>SUM(AS4:AZ4)+BK4+BL4</f>
-        <v>520.27386164750192</v>
+        <v>1113.1414478988468</v>
       </c>
       <c r="AR4" s="5">
         <f>AP4-AQ4</f>
@@ -1295,23 +1320,23 @@
       </c>
       <c r="AS4" s="5">
         <f>E4/G4*X4</f>
-        <v>0</v>
+        <v>412.75246205135954</v>
       </c>
       <c r="AT4" s="1">
         <f>F4/G4*W4</f>
-        <v>0</v>
+        <v>41.162216940662823</v>
       </c>
       <c r="AU4" s="1">
-        <f>1/G4*T4</f>
-        <v>193.26004546602891</v>
+        <f>1/G4*(O4+P4)</f>
+        <v>985.04107428117129</v>
       </c>
       <c r="AV4" s="1">
         <f>H4/G4*AF4*-1</f>
-        <v>0</v>
+        <v>-6.5982742166693766</v>
       </c>
       <c r="AW4" s="1">
         <f>I4/G4*Z4</f>
-        <v>0</v>
+        <v>-646.22984733915064</v>
       </c>
       <c r="AX4" s="1">
         <f>K4/G4/(0.9*8760)</f>
@@ -1470,31 +1495,55 @@
       <c r="O5" s="16">
         <v>122.135409</v>
       </c>
-      <c r="P5" s="16"/>
-      <c r="Q5" s="16"/>
-      <c r="R5" s="16"/>
-      <c r="S5" s="16"/>
+      <c r="P5" s="16">
+        <v>-10.071578000000001</v>
+      </c>
+      <c r="Q5" s="16">
+        <v>73.297528</v>
+      </c>
+      <c r="R5" s="16">
+        <v>77.158259999999999</v>
+      </c>
+      <c r="S5" s="16">
+        <v>59.694023999999999</v>
+      </c>
       <c r="T5" s="11">
         <v>21.986353300000001</v>
       </c>
       <c r="U5" s="17"/>
       <c r="V5" s="17"/>
-      <c r="W5" s="16"/>
-      <c r="X5" s="16"/>
+      <c r="W5" s="16">
+        <v>26.556269</v>
+      </c>
+      <c r="X5" s="16">
+        <v>8.6278919999999992</v>
+      </c>
       <c r="Y5" s="16"/>
-      <c r="Z5" s="17"/>
-      <c r="AA5" s="17"/>
+      <c r="Z5" s="17">
+        <v>-96.133976000000004</v>
+      </c>
+      <c r="AA5" s="17">
+        <v>-96.133976000000004</v>
+      </c>
       <c r="AB5" s="17"/>
       <c r="AC5" s="17"/>
       <c r="AD5" s="17"/>
       <c r="AE5" s="17"/>
-      <c r="AF5" s="16"/>
-      <c r="AG5" s="16"/>
-      <c r="AH5" s="16"/>
-      <c r="AI5" s="16"/>
+      <c r="AF5" s="16">
+        <v>4.7546840000000001</v>
+      </c>
+      <c r="AG5" s="16">
+        <v>-0.13628299999999999</v>
+      </c>
+      <c r="AH5" s="16">
+        <v>576.81126900000004</v>
+      </c>
+      <c r="AI5" s="16">
+        <v>576.81126900000004</v>
+      </c>
       <c r="AK5" s="1" t="str">
         <f>B5</f>
-        <v>Synthetic_Ethylene_CCS_90</v>
+        <v>SE_Synthetic_Ethylene_CCS_90</v>
       </c>
       <c r="AL5" s="1" t="str">
         <f>C5</f>
@@ -1502,11 +1551,11 @@
       </c>
       <c r="AM5" s="12">
         <f>SUM(AS5:AZ5)+BB5+BC5</f>
-        <v>491.18316495374813</v>
+        <v>1030.9511213412507</v>
       </c>
       <c r="AN5" s="12">
         <f>SUM(AS5:AZ5)+BE5+BF5</f>
-        <v>491.18316495374813</v>
+        <v>1030.9511213412507</v>
       </c>
       <c r="AO5" s="5">
         <f>AM5-AN5</f>
@@ -1514,11 +1563,11 @@
       </c>
       <c r="AP5" s="12">
         <f>SUM(AS5:AZ5)+BH5+BI5</f>
-        <v>538.67601721659707</v>
+        <v>1078.4439736040995</v>
       </c>
       <c r="AQ5" s="12">
         <f>SUM(AS5:AZ5)+BK5+BL5</f>
-        <v>538.67601721659707</v>
+        <v>1078.4439736040995</v>
       </c>
       <c r="AR5" s="5">
         <f>AP5-AQ5</f>
@@ -1526,23 +1575,23 @@
       </c>
       <c r="AS5" s="5">
         <f>E5/G5*X5</f>
-        <v>0</v>
+        <v>412.75246220347435</v>
       </c>
       <c r="AT5" s="1">
         <f>F5/G5*W5</f>
-        <v>0</v>
+        <v>52.467220678186571</v>
       </c>
       <c r="AU5" s="1">
-        <f>1/G5*T5</f>
-        <v>177.53998910942985</v>
+        <f>1/G5*(O5+P5)</f>
+        <v>904.91638444202511</v>
       </c>
       <c r="AV5" s="1">
         <f>H5/G5*AF5*-1</f>
-        <v>0</v>
+        <v>-6.598274219868598</v>
       </c>
       <c r="AW5" s="1">
         <f>I5/G5*Z5</f>
-        <v>0</v>
+        <v>-646.22984760688507</v>
       </c>
       <c r="AX5" s="1">
         <f>K5/G5/(0.9*8760)</f>
@@ -5527,422 +5576,436 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F389C78-28A3-1242-8015-D6A42DDB2312}">
-  <dimension ref="B2:AL5"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="B2:T5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="2.6640625" customWidth="1"/>
     <col min="2" max="2" width="26.5" customWidth="1"/>
-    <col min="3" max="3" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17.83203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.83203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="17.1640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.5" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="14.5" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.83203125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="5.1640625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="9.1640625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="10.5" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="13.1640625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="2.33203125" customWidth="1"/>
-    <col min="21" max="21" width="14.5" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="15.33203125" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="17.83203125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="15.83203125" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="17.1640625" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="14" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="12.5" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="14.5" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="10.83203125" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="15.6640625" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="5.6640625" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="9.1640625" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="10.5" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="13.1640625" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="2.6640625" customWidth="1"/>
-    <col min="36" max="36" width="11.83203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.83203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.83203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.1640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.5" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.5" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.83203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="5.1640625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.1640625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="13.1640625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="2.6640625" customWidth="1"/>
+    <col min="18" max="18" width="11.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:38" x14ac:dyDescent="0.2">
+    <row r="2" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B2" s="21" t="s">
-        <v>90</v>
-      </c>
-      <c r="S2" s="21" t="s">
-        <v>91</v>
-      </c>
-      <c r="AJ2" s="24" t="s">
+        <v>89</v>
+      </c>
+      <c r="R2" s="24" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="2:38" ht="32" x14ac:dyDescent="0.2">
+    <row r="3" spans="2:20" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B3" s="4" t="s">
         <v>48</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="J3" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="K3" s="4" t="s">
         <v>59</v>
       </c>
+      <c r="K3" s="22" t="s">
+        <v>61</v>
+      </c>
       <c r="L3" s="22" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="M3" s="22" t="s">
-        <v>62</v>
-      </c>
-      <c r="N3" s="22" t="s">
         <v>60</v>
       </c>
+      <c r="N3" s="23" t="s">
+        <v>50</v>
+      </c>
       <c r="O3" s="23" t="s">
-        <v>50</v>
+        <v>90</v>
       </c>
       <c r="P3" s="23" t="s">
-        <v>89</v>
-      </c>
-      <c r="Q3" s="23" t="s">
-        <v>94</v>
-      </c>
-      <c r="S3" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="T3" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="U3" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="V3" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="W3" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="X3" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="Y3" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="Z3" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="AA3" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="AB3" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="AC3" s="22" t="s">
-        <v>61</v>
-      </c>
-      <c r="AD3" s="22" t="s">
-        <v>62</v>
-      </c>
-      <c r="AE3" s="22" t="s">
-        <v>60</v>
-      </c>
-      <c r="AF3" s="23" t="s">
-        <v>50</v>
-      </c>
-      <c r="AG3" s="23" t="s">
-        <v>89</v>
-      </c>
-      <c r="AH3" s="23" t="s">
-        <v>94</v>
-      </c>
-      <c r="AJ3" t="s">
+        <v>91</v>
+      </c>
+      <c r="R3" t="s">
         <v>92</v>
       </c>
-      <c r="AK3">
+      <c r="S3">
         <v>45.6</v>
       </c>
-      <c r="AL3" t="s">
+      <c r="T3" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="4" spans="2:38" x14ac:dyDescent="0.2">
+    <row r="4" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B4" t="str">
         <f>lc_detailed!AK4</f>
-        <v>Synthetic_Ethylene_Non_CCS</v>
-      </c>
-      <c r="C4" t="str">
-        <f>lc_detailed!AL4</f>
-        <v>CO2Captured</v>
+        <v>SE_Synthetic_Ethylene_Non_CCS</v>
+      </c>
+      <c r="C4" s="25">
+        <f>lc_detailed!AS4/$S$3</f>
+        <v>9.0515890800736738</v>
       </c>
       <c r="D4" s="25">
-        <f>lc_detailed!AS4/$AK$3</f>
+        <f>lc_detailed!AT4/$S$3</f>
+        <v>0.9026801960671671</v>
+      </c>
+      <c r="E4" s="25">
+        <f>lc_detailed!AU4/$S$3</f>
+        <v>21.601777944762528</v>
+      </c>
+      <c r="F4" s="25">
+        <f>lc_detailed!AV4/$S$3</f>
+        <v>-0.1446989959795916</v>
+      </c>
+      <c r="G4" s="25">
+        <f>lc_detailed!AW4/$S$3</f>
+        <v>-14.171707178490145</v>
+      </c>
+      <c r="H4" s="25">
+        <f>lc_detailed!AX4/$S$3</f>
+        <v>4.2600965636830308</v>
+      </c>
+      <c r="I4" s="25">
+        <f>lc_detailed!AY4/$S$3</f>
+        <v>2.3433206377337097</v>
+      </c>
+      <c r="J4" s="25">
+        <f>lc_detailed!AZ4/$S$3</f>
+        <v>0.56793841659801814</v>
+      </c>
+      <c r="K4" s="25">
+        <f>lc_detailed!BH4/$S$3</f>
         <v>0</v>
       </c>
-      <c r="E4" s="25">
-        <f>lc_detailed!AT4/$AK$3</f>
+      <c r="L4" s="25">
+        <f>lc_detailed!BI4/$S$3</f>
         <v>0</v>
       </c>
-      <c r="F4" s="25">
-        <f>lc_detailed!AU4/$AK$3</f>
-        <v>4.2381588917988795</v>
-      </c>
-      <c r="G4" s="25">
-        <f>lc_detailed!AV4/$AK$3</f>
-        <v>0</v>
-      </c>
-      <c r="H4" s="25">
-        <f>lc_detailed!AW4/$AK$3</f>
-        <v>0</v>
-      </c>
-      <c r="I4" s="25">
-        <f>lc_detailed!AX4/$AK$3</f>
-        <v>4.2600965636830308</v>
-      </c>
-      <c r="J4" s="25">
-        <f>lc_detailed!AY4/$AK$3</f>
-        <v>2.3433206377337097</v>
-      </c>
-      <c r="K4" s="25">
-        <f>lc_detailed!AZ4/$AK$3</f>
-        <v>0.56793841659801814</v>
-      </c>
-      <c r="L4" s="25">
-        <f>lc_detailed!BH4/$AK$3</f>
-        <v>0</v>
-      </c>
       <c r="M4" s="25">
-        <f>lc_detailed!BI4/$AK$3</f>
-        <v>0</v>
-      </c>
-      <c r="N4" s="25">
         <f>lc_detailed!BG4</f>
         <v>0</v>
       </c>
+      <c r="N4" s="25">
+        <f>lc_detailed!AP4</f>
+        <v>1113.1414478988468</v>
+      </c>
       <c r="O4" s="25">
-        <f>lc_detailed!AP4</f>
-        <v>520.27386164750192</v>
+        <f>N4/$S$3</f>
+        <v>24.410996664448394</v>
       </c>
       <c r="P4" s="25">
-        <f>O4/$AK$3</f>
-        <v>11.409514509813638</v>
-      </c>
-      <c r="Q4" s="25">
-        <f>SUM(D4:M4)</f>
-        <v>11.409514509813638</v>
-      </c>
-      <c r="S4" t="str">
+        <f>SUM(C4:L4)</f>
+        <v>24.41099666444839</v>
+      </c>
+    </row>
+    <row r="5" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B5" t="str">
+        <f>lc_detailed!AK5</f>
+        <v>SE_Synthetic_Ethylene_CCS_90</v>
+      </c>
+      <c r="C5" s="25">
+        <f>lc_detailed!AS5/$S$3</f>
+        <v>9.0515890834095245</v>
+      </c>
+      <c r="D5" s="25">
+        <f>lc_detailed!AT5/$S$3</f>
+        <v>1.1505969446970739</v>
+      </c>
+      <c r="E5" s="25">
+        <f>lc_detailed!AU5/$S$3</f>
+        <v>19.84465755355318</v>
+      </c>
+      <c r="F5" s="25">
+        <f>lc_detailed!AV5/$S$3</f>
+        <v>-0.14469899604974995</v>
+      </c>
+      <c r="G5" s="25">
+        <f>lc_detailed!AW5/$S$3</f>
+        <v>-14.171707184361514</v>
+      </c>
+      <c r="H5" s="25">
+        <f>lc_detailed!AX5/$S$3</f>
+        <v>4.705568157602146</v>
+      </c>
+      <c r="I5" s="25">
+        <f>lc_detailed!AY5/$S$3</f>
+        <v>2.5867547372464941</v>
+      </c>
+      <c r="J5" s="25">
+        <f>lc_detailed!AZ5/$S$3</f>
+        <v>0.62732684434362407</v>
+      </c>
+      <c r="K5" s="25">
+        <f>lc_detailed!BH5/$S$3</f>
+        <v>0</v>
+      </c>
+      <c r="L5" s="25">
+        <f>lc_detailed!BI5/$S$3</f>
+        <v>0</v>
+      </c>
+      <c r="M5" s="25">
+        <f>lc_detailed!BG5</f>
+        <v>0</v>
+      </c>
+      <c r="N5" s="25">
+        <f>lc_detailed!AP5</f>
+        <v>1078.4439736040995</v>
+      </c>
+      <c r="O5" s="25">
+        <f>N5/$S$3</f>
+        <v>23.650087140440778</v>
+      </c>
+      <c r="P5" s="25">
+        <f>SUM(C5:L5)</f>
+        <v>23.650087140440778</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="B2:T5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="2.33203125" customWidth="1"/>
+    <col min="2" max="2" width="13.5" customWidth="1"/>
+    <col min="3" max="3" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.1640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.83203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15.83203125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.5" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="13" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="2.33203125" customWidth="1"/>
+    <col min="18" max="18" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="6" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="12.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B2" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="R2" s="24" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="2:20" ht="48" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B3" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="J3" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="K3" s="22" t="s">
+        <v>61</v>
+      </c>
+      <c r="L3" s="22" t="s">
+        <v>62</v>
+      </c>
+      <c r="M3" s="22" t="s">
+        <v>60</v>
+      </c>
+      <c r="N3" s="23" t="s">
+        <v>50</v>
+      </c>
+      <c r="O3" s="23" t="s">
+        <v>90</v>
+      </c>
+      <c r="P3" s="23" t="s">
+        <v>91</v>
+      </c>
+      <c r="R3" t="s">
+        <v>92</v>
+      </c>
+      <c r="S3">
+        <v>45.6</v>
+      </c>
+      <c r="T3" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="4" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B4" t="str">
         <f>lc_detailed!AK4</f>
-        <v>Synthetic_Ethylene_Non_CCS</v>
-      </c>
-      <c r="T4" t="str">
-        <f>lc_detailed!AL4</f>
-        <v>CO2Captured</v>
-      </c>
-      <c r="U4" s="25">
-        <f>lc_detailed!AS4/$AK$3</f>
+        <v>SE_Synthetic_Ethylene_Non_CCS</v>
+      </c>
+      <c r="C4" s="25">
+        <f>lc_detailed!AS4/$S$3</f>
+        <v>9.0515890800736738</v>
+      </c>
+      <c r="D4" s="25">
+        <f>lc_detailed!AT4/$S$3</f>
+        <v>0.9026801960671671</v>
+      </c>
+      <c r="E4" s="25">
+        <f>lc_detailed!AU4/$S$3</f>
+        <v>21.601777944762528</v>
+      </c>
+      <c r="F4" s="25">
+        <f>lc_detailed!AV4/$S$3</f>
+        <v>-0.1446989959795916</v>
+      </c>
+      <c r="G4" s="25">
+        <f>lc_detailed!AW4/$S$3</f>
+        <v>-14.171707178490145</v>
+      </c>
+      <c r="H4" s="25">
+        <f>lc_detailed!AX4/$S$3</f>
+        <v>4.2600965636830308</v>
+      </c>
+      <c r="I4" s="25">
+        <f>lc_detailed!AY4/$S$3</f>
+        <v>2.3433206377337097</v>
+      </c>
+      <c r="J4" s="25">
+        <f>lc_detailed!AZ4/$S$3</f>
+        <v>0.56793841659801814</v>
+      </c>
+      <c r="K4" s="25">
+        <f>lc_detailed!BB4/$S$3</f>
         <v>0</v>
       </c>
-      <c r="V4" s="25">
-        <f>lc_detailed!AT4/$AK$3</f>
-        <v>0</v>
-      </c>
-      <c r="W4" s="25">
-        <f>lc_detailed!AU4/$AK$3</f>
-        <v>4.2381588917988795</v>
-      </c>
-      <c r="X4" s="25">
-        <f>lc_detailed!AV4/$AK$3</f>
-        <v>0</v>
-      </c>
-      <c r="Y4" s="25">
-        <f>lc_detailed!AW4/$AK$3</f>
-        <v>0</v>
-      </c>
-      <c r="Z4" s="25">
-        <f>lc_detailed!AX4/$AK$3</f>
-        <v>4.2600965636830308</v>
-      </c>
-      <c r="AA4" s="25">
-        <f>lc_detailed!AY4/$AK$3</f>
-        <v>2.3433206377337097</v>
-      </c>
-      <c r="AB4" s="25">
-        <f>lc_detailed!AZ4/$AK$3</f>
-        <v>0.56793841659801814</v>
-      </c>
-      <c r="AC4" s="25">
-        <f>lc_detailed!BB4/$AK$3</f>
-        <v>0</v>
-      </c>
-      <c r="AD4" s="25">
-        <f>lc_detailed!BC4/$AK$3</f>
+      <c r="L4" s="25">
+        <f>lc_detailed!BC4/$S$3</f>
         <v>-0.95679196939630118</v>
       </c>
-      <c r="AE4" s="25">
+      <c r="M4" s="25">
         <f>lc_detailed!BD4</f>
         <v>-0.35722411839199997</v>
       </c>
-      <c r="AF4" s="25">
+      <c r="N4" s="25">
         <f>lc_detailed!AM4</f>
-        <v>476.64414784303057</v>
-      </c>
-      <c r="AG4" s="25">
-        <f>AF4/$AK$3</f>
-        <v>10.452722540417337</v>
-      </c>
-      <c r="AH4" s="25">
-        <f>SUM(U4:AD4)</f>
-        <v>10.452722540417337</v>
-      </c>
-    </row>
-    <row r="5" spans="2:38" x14ac:dyDescent="0.2">
+        <v>1069.5117340943755</v>
+      </c>
+      <c r="O4" s="25">
+        <f>N4/$S$3</f>
+        <v>23.454204695052091</v>
+      </c>
+      <c r="P4" s="25">
+        <f>SUM(C4:L4)</f>
+        <v>23.454204695052088</v>
+      </c>
+    </row>
+    <row r="5" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B5" t="str">
         <f>lc_detailed!AK5</f>
-        <v>Synthetic_Ethylene_CCS_90</v>
-      </c>
-      <c r="C5" t="str">
-        <f>lc_detailed!AL5</f>
-        <v>CO2Captured</v>
+        <v>SE_Synthetic_Ethylene_CCS_90</v>
+      </c>
+      <c r="C5" s="25">
+        <f>lc_detailed!AS5/$S$3</f>
+        <v>9.0515890834095245</v>
       </c>
       <c r="D5" s="25">
-        <f>lc_detailed!AS5/$AK$3</f>
+        <f>lc_detailed!AT5/$S$3</f>
+        <v>1.1505969446970739</v>
+      </c>
+      <c r="E5" s="25">
+        <f>lc_detailed!AU5/$S$3</f>
+        <v>19.84465755355318</v>
+      </c>
+      <c r="F5" s="25">
+        <f>lc_detailed!AV5/$S$3</f>
+        <v>-0.14469899604974995</v>
+      </c>
+      <c r="G5" s="25">
+        <f>lc_detailed!AW5/$S$3</f>
+        <v>-14.171707184361514</v>
+      </c>
+      <c r="H5" s="25">
+        <f>lc_detailed!AX5/$S$3</f>
+        <v>4.705568157602146</v>
+      </c>
+      <c r="I5" s="25">
+        <f>lc_detailed!AY5/$S$3</f>
+        <v>2.5867547372464941</v>
+      </c>
+      <c r="J5" s="25">
+        <f>lc_detailed!AZ5/$S$3</f>
+        <v>0.62732684434362407</v>
+      </c>
+      <c r="K5" s="25">
+        <f>lc_detailed!BB5/$S$3</f>
         <v>0</v>
       </c>
-      <c r="E5" s="25">
-        <f>lc_detailed!AT5/$AK$3</f>
-        <v>0</v>
-      </c>
-      <c r="F5" s="25">
-        <f>lc_detailed!AU5/$AK$3</f>
-        <v>3.893420813803286</v>
-      </c>
-      <c r="G5" s="25">
-        <f>lc_detailed!AV5/$AK$3</f>
-        <v>0</v>
-      </c>
-      <c r="H5" s="25">
-        <f>lc_detailed!AW5/$AK$3</f>
-        <v>0</v>
-      </c>
-      <c r="I5" s="25">
-        <f>lc_detailed!AX5/$AK$3</f>
-        <v>4.705568157602146</v>
-      </c>
-      <c r="J5" s="25">
-        <f>lc_detailed!AY5/$AK$3</f>
-        <v>2.5867547372464941</v>
-      </c>
-      <c r="K5" s="25">
-        <f>lc_detailed!AZ5/$AK$3</f>
-        <v>0.62732684434362407</v>
-      </c>
       <c r="L5" s="25">
-        <f>lc_detailed!BH5/$AK$3</f>
-        <v>0</v>
+        <f>lc_detailed!BC5/$S$3</f>
+        <v>-1.0415099180449323</v>
       </c>
       <c r="M5" s="25">
-        <f>lc_detailed!BI5/$AK$3</f>
-        <v>0</v>
-      </c>
-      <c r="N5" s="25">
-        <f>lc_detailed!BG5</f>
-        <v>0</v>
-      </c>
-      <c r="O5" s="25">
-        <f>lc_detailed!AP5</f>
-        <v>538.67601721659707</v>
-      </c>
-      <c r="P5" s="25">
-        <f>O5/$AK$3</f>
-        <v>11.81307055299555</v>
-      </c>
-      <c r="Q5" s="25">
-        <f>SUM(D5:M5)</f>
-        <v>11.813070552995551</v>
-      </c>
-      <c r="S5" t="str">
-        <f>lc_detailed!AK5</f>
-        <v>Synthetic_Ethylene_CCS_90</v>
-      </c>
-      <c r="T5" t="str">
-        <f>lc_detailed!AL5</f>
-        <v>CO2Captured</v>
-      </c>
-      <c r="U5" s="25">
-        <f>lc_detailed!AS5/$AK$3</f>
-        <v>0</v>
-      </c>
-      <c r="V5" s="25">
-        <f>lc_detailed!AT5/$AK$3</f>
-        <v>0</v>
-      </c>
-      <c r="W5" s="25">
-        <f>lc_detailed!AU5/$AK$3</f>
-        <v>3.893420813803286</v>
-      </c>
-      <c r="X5" s="25">
-        <f>lc_detailed!AV5/$AK$3</f>
-        <v>0</v>
-      </c>
-      <c r="Y5" s="25">
-        <f>lc_detailed!AW5/$AK$3</f>
-        <v>0</v>
-      </c>
-      <c r="Z5" s="25">
-        <f>lc_detailed!AX5/$AK$3</f>
-        <v>4.705568157602146</v>
-      </c>
-      <c r="AA5" s="25">
-        <f>lc_detailed!AY5/$AK$3</f>
-        <v>2.5867547372464941</v>
-      </c>
-      <c r="AB5" s="25">
-        <f>lc_detailed!AZ5/$AK$3</f>
-        <v>0.62732684434362407</v>
-      </c>
-      <c r="AC5" s="25">
-        <f>lc_detailed!BB5/$AK$3</f>
-        <v>0</v>
-      </c>
-      <c r="AD5" s="25">
-        <f>lc_detailed!BC5/$AK$3</f>
-        <v>-1.0415099180449323</v>
-      </c>
-      <c r="AE5" s="25">
         <f>lc_detailed!BD5</f>
         <v>-0.38885408131599997</v>
       </c>
-      <c r="AF5" s="25">
+      <c r="N5" s="25">
         <f>lc_detailed!AM5</f>
-        <v>491.18316495374813</v>
-      </c>
-      <c r="AG5" s="25">
-        <f>AF5/$AK$3</f>
-        <v>10.771560634950617</v>
-      </c>
-      <c r="AH5" s="25">
-        <f>SUM(U5:AD5)</f>
-        <v>10.771560634950619</v>
+        <v>1030.9511213412507</v>
+      </c>
+      <c r="O5" s="25">
+        <f>N5/$S$3</f>
+        <v>22.608577222395848</v>
+      </c>
+      <c r="P5" s="25">
+        <f>SUM(C5:L5)</f>
+        <v>22.608577222395844</v>
       </c>
     </row>
   </sheetData>

</xml_diff>